<commit_message>
add new measurement and finish up drawing 011 brass needle valve
</commit_message>
<xml_diff>
--- a/Measurements/17016PP brush cutter blade bolt/17016PP.xlsx
+++ b/Measurements/17016PP brush cutter blade bolt/17016PP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\17016PP brush cutter blade bolt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B0498E-D4F4-4722-951F-D55A7A7EF692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B042B102-3C0A-4240-96FC-53E549E39532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -200,7 +200,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -227,21 +227,6 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
       <right style="double">
         <color auto="1"/>
       </right>
@@ -461,19 +446,6 @@
     </border>
     <border>
       <left style="double">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color auto="1"/>
       </left>
       <right style="thin">
@@ -627,26 +599,26 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -655,13 +627,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -670,10 +642,10 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -685,130 +657,112 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2621,23 +2575,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:20" ht="30" customHeight="1">
-      <c r="B1" s="54" t="s">
+      <c r="B1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="54"/>
-      <c r="O1" s="54"/>
-      <c r="P1" s="54"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
       <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="2:20" ht="26.45" customHeight="1" thickBot="1">
@@ -2710,42 +2664,42 @@
       <c r="B4" s="7">
         <v>1</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="47">
-        <v>2.7585000000000002</v>
-      </c>
-      <c r="F4" s="52">
+      <c r="E4" s="41">
+        <v>2.7490000000000001</v>
+      </c>
+      <c r="F4" s="46">
         <v>0.91</v>
       </c>
-      <c r="G4" s="52">
+      <c r="G4" s="46">
         <v>0.53300000000000003</v>
       </c>
-      <c r="H4" s="52">
+      <c r="H4" s="46">
         <v>1.496</v>
       </c>
-      <c r="I4" s="52">
+      <c r="I4" s="46">
         <v>1.125</v>
       </c>
-      <c r="J4" s="55">
+      <c r="J4" s="46">
         <v>2.3915000000000002</v>
       </c>
-      <c r="K4" s="55">
+      <c r="K4" s="46">
         <v>1.486</v>
       </c>
-      <c r="L4" s="58">
+      <c r="L4" s="48">
         <v>7.0250000000000007E-2</v>
       </c>
-      <c r="M4" s="58">
+      <c r="M4" s="48">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="28"/>
+      <c r="N4" s="52"/>
+      <c r="O4" s="52"/>
+      <c r="P4" s="25"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="21"/>
     </row>
@@ -2753,42 +2707,42 @@
       <c r="B5" s="7">
         <v>2</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="48" t="s">
+      <c r="D5" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="47">
-        <v>2.7519999999999998</v>
-      </c>
-      <c r="F5" s="47">
+      <c r="E5" s="41">
+        <v>2.7429999999999999</v>
+      </c>
+      <c r="F5" s="41">
         <v>0.89849999999999997</v>
       </c>
-      <c r="G5" s="47">
+      <c r="G5" s="41">
         <v>0.53800000000000003</v>
       </c>
-      <c r="H5" s="52">
+      <c r="H5" s="46">
         <v>1.494</v>
       </c>
-      <c r="I5" s="47">
+      <c r="I5" s="41">
         <v>1.1240000000000001</v>
       </c>
-      <c r="J5" s="56">
+      <c r="J5" s="41">
         <v>2.3915000000000002</v>
       </c>
-      <c r="K5" s="56">
+      <c r="K5" s="41">
         <v>1.4870000000000001</v>
       </c>
-      <c r="L5" s="59">
+      <c r="L5" s="49">
         <v>7.0250000000000007E-2</v>
       </c>
-      <c r="M5" s="58">
+      <c r="M5" s="48">
         <v>6.9500000000000006E-2</v>
       </c>
-      <c r="N5" s="29"/>
-      <c r="O5" s="25"/>
-      <c r="P5" s="30"/>
+      <c r="N5" s="53"/>
+      <c r="O5" s="52"/>
+      <c r="P5" s="26"/>
       <c r="Q5" s="22"/>
       <c r="R5" s="23"/>
     </row>
@@ -2796,42 +2750,42 @@
       <c r="B6" s="7">
         <v>3</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="47">
-        <v>2.7675000000000001</v>
-      </c>
-      <c r="F6" s="47">
+      <c r="E6" s="41">
+        <v>2.7480000000000002</v>
+      </c>
+      <c r="F6" s="41">
         <v>0.89949999999999997</v>
       </c>
-      <c r="G6" s="47">
+      <c r="G6" s="41">
         <v>0.54749999999999999</v>
       </c>
-      <c r="H6" s="52">
+      <c r="H6" s="46">
         <v>1.4950000000000001</v>
       </c>
-      <c r="I6" s="47">
+      <c r="I6" s="41">
         <v>1.1214999999999999</v>
       </c>
-      <c r="J6" s="56">
+      <c r="J6" s="41">
         <v>2.3875000000000002</v>
       </c>
-      <c r="K6" s="56">
+      <c r="K6" s="41">
         <v>1.484</v>
       </c>
-      <c r="L6" s="56">
+      <c r="L6" s="41">
         <v>6.0449999999999997E-2</v>
       </c>
-      <c r="M6" s="58">
+      <c r="M6" s="48">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="N6" s="29"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="30"/>
+      <c r="N6" s="53"/>
+      <c r="O6" s="52"/>
+      <c r="P6" s="26"/>
       <c r="Q6" s="22"/>
       <c r="R6" s="23"/>
     </row>
@@ -2839,42 +2793,42 @@
       <c r="B7" s="7">
         <v>4</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="47">
-        <v>2.75</v>
-      </c>
-      <c r="F7" s="47">
+      <c r="E7" s="41">
+        <v>2.7559999999999998</v>
+      </c>
+      <c r="F7" s="41">
         <v>0.89400000000000002</v>
       </c>
-      <c r="G7" s="47">
+      <c r="G7" s="41">
         <v>0.55000000000000004</v>
       </c>
-      <c r="H7" s="52">
+      <c r="H7" s="46">
         <v>1.496</v>
       </c>
-      <c r="I7" s="47">
+      <c r="I7" s="41">
         <v>1.125</v>
       </c>
-      <c r="J7" s="56">
+      <c r="J7" s="41">
         <v>2.39</v>
       </c>
-      <c r="K7" s="56">
+      <c r="K7" s="41">
         <v>1.494</v>
       </c>
-      <c r="L7" s="59">
+      <c r="L7" s="49">
         <v>7.1499999999999994E-2</v>
       </c>
-      <c r="M7" s="58">
+      <c r="M7" s="48">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N7" s="29"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="30"/>
+      <c r="N7" s="53"/>
+      <c r="O7" s="52"/>
+      <c r="P7" s="26"/>
       <c r="Q7" s="22"/>
       <c r="R7" s="23"/>
     </row>
@@ -2882,66 +2836,66 @@
       <c r="B8" s="15">
         <v>5</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="50" t="s">
+      <c r="D8" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="51">
-        <v>2.7574999999999998</v>
-      </c>
-      <c r="F8" s="51">
+      <c r="E8" s="45">
+        <v>2.742</v>
+      </c>
+      <c r="F8" s="45">
         <v>0.89349999999999996</v>
       </c>
-      <c r="G8" s="53">
+      <c r="G8" s="47">
         <v>0.54400000000000004</v>
       </c>
-      <c r="H8" s="53">
+      <c r="H8" s="47">
         <v>1.4950000000000001</v>
       </c>
-      <c r="I8" s="53">
+      <c r="I8" s="47">
         <v>1.1225000000000001</v>
       </c>
-      <c r="J8" s="57">
+      <c r="J8" s="47">
         <v>2.3915000000000002</v>
       </c>
-      <c r="K8" s="57">
+      <c r="K8" s="47">
         <v>1.4850000000000001</v>
       </c>
-      <c r="L8" s="60">
+      <c r="L8" s="50">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="M8" s="60">
+      <c r="M8" s="50">
         <v>6.8500000000000005E-2</v>
       </c>
-      <c r="N8" s="31"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="33"/>
+      <c r="N8" s="54"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="27"/>
       <c r="Q8" s="15"/>
       <c r="R8" s="24"/>
     </row>
     <row r="9" spans="2:20" ht="6.75" customHeight="1" thickTop="1"/>
     <row r="10" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B10" s="34"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="36"/>
-      <c r="P10" s="37"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="30"/>
+      <c r="P10" s="31"/>
       <c r="Q10" s="8"/>
     </row>
     <row r="11" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B11" s="38"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="8"/>
@@ -2955,14 +2909,14 @@
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
-      <c r="P11" s="39"/>
+      <c r="P11" s="33"/>
       <c r="Q11" s="8"/>
       <c r="T11" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="12" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B12" s="38"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
       <c r="E12" s="8"/>
@@ -2976,11 +2930,11 @@
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
-      <c r="P12" s="39"/>
+      <c r="P12" s="33"/>
       <c r="Q12" s="8"/>
     </row>
     <row r="13" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B13" s="38"/>
+      <c r="B13" s="32"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="8"/>
@@ -2994,11 +2948,11 @@
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
-      <c r="P13" s="39"/>
+      <c r="P13" s="33"/>
       <c r="Q13" s="8"/>
     </row>
     <row r="14" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B14" s="38"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="8"/>
@@ -3012,11 +2966,11 @@
       <c r="M14" s="8"/>
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
-      <c r="P14" s="39"/>
+      <c r="P14" s="33"/>
       <c r="Q14" s="8"/>
     </row>
     <row r="15" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B15" s="38"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
       <c r="E15" s="8"/>
@@ -3030,11 +2984,11 @@
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
-      <c r="P15" s="39"/>
+      <c r="P15" s="33"/>
       <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="2:20" ht="20.100000000000001" customHeight="1">
-      <c r="B16" s="38"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="8"/>
@@ -3048,11 +3002,11 @@
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
-      <c r="P16" s="39"/>
+      <c r="P16" s="33"/>
       <c r="Q16" s="8"/>
     </row>
     <row r="17" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B17" s="38"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="8"/>
@@ -3066,11 +3020,11 @@
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
       <c r="O17" s="8"/>
-      <c r="P17" s="39"/>
+      <c r="P17" s="33"/>
       <c r="Q17" s="8"/>
     </row>
     <row r="18" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B18" s="38"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="8"/>
@@ -3084,14 +3038,14 @@
       <c r="M18" s="8"/>
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
-      <c r="P18" s="39"/>
+      <c r="P18" s="33"/>
       <c r="Q18" s="8"/>
       <c r="W18" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="19" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B19" s="38"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="8"/>
@@ -3105,11 +3059,11 @@
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
-      <c r="P19" s="39"/>
+      <c r="P19" s="33"/>
       <c r="Q19" s="8"/>
     </row>
     <row r="20" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B20" s="38"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="8"/>
@@ -3123,11 +3077,11 @@
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
-      <c r="P20" s="39"/>
+      <c r="P20" s="33"/>
       <c r="Q20" s="8"/>
     </row>
     <row r="21" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B21" s="38"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
       <c r="E21" s="8"/>
@@ -3141,12 +3095,12 @@
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
-      <c r="P21" s="39"/>
+      <c r="P21" s="33"/>
       <c r="Q21" s="8"/>
     </row>
     <row r="22" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B22" s="40"/>
-      <c r="C22" s="41"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="35"/>
       <c r="D22" s="13"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
@@ -3159,11 +3113,11 @@
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
-      <c r="P22" s="39"/>
+      <c r="P22" s="33"/>
       <c r="Q22" s="8"/>
     </row>
     <row r="23" spans="2:23" ht="20.100000000000001" customHeight="1">
-      <c r="B23" s="38"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="8"/>
@@ -3177,11 +3131,11 @@
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
-      <c r="P23" s="39"/>
+      <c r="P23" s="33"/>
       <c r="Q23" s="8"/>
     </row>
     <row r="24" spans="2:23">
-      <c r="B24" s="38"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
       <c r="E24" s="8"/>
@@ -3195,11 +3149,11 @@
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
-      <c r="P24" s="39"/>
+      <c r="P24" s="33"/>
       <c r="Q24" s="8"/>
     </row>
     <row r="25" spans="2:23">
-      <c r="B25" s="38"/>
+      <c r="B25" s="32"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
       <c r="E25" s="8"/>
@@ -3213,25 +3167,25 @@
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>
       <c r="O25" s="8"/>
-      <c r="P25" s="39"/>
+      <c r="P25" s="33"/>
       <c r="Q25" s="8"/>
     </row>
     <row r="26" spans="2:23">
-      <c r="B26" s="42"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="44"/>
-      <c r="P26" s="45"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="38"/>
+      <c r="K26" s="38"/>
+      <c r="L26" s="38"/>
+      <c r="M26" s="38"/>
+      <c r="N26" s="38"/>
+      <c r="O26" s="38"/>
+      <c r="P26" s="39"/>
       <c r="Q26" s="8"/>
     </row>
     <row r="27" spans="2:23">

</xml_diff>